<commit_message>
new measurements of the test-PCB: - Best-fit curve - Buffer LT6203 - Alternatives for input buffer
</commit_message>
<xml_diff>
--- a/-5V_PCB/Measurements/ADC_LTC2311-16_-5VTestingPCB_InternalPowerSupply_5.2Vrails.xlsx
+++ b/-5V_PCB/Measurements/ADC_LTC2311-16_-5VTestingPCB_InternalPowerSupply_5.2Vrails.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\simon\Desktop\Bachelorarbeit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1868FC1D-5728-4740-83CC-CF93E9EB8065}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5878F7CF-ADB8-4ECE-AB66-8335DEBA01F6}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{495E718F-06B1-4643-B7E0-98C6B6E2ABE9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{495E718F-06B1-4643-B7E0-98C6B6E2ABE9}"/>
   </bookViews>
   <sheets>
     <sheet name="Single-ended" sheetId="3" r:id="rId1"/>
@@ -1719,7 +1719,7 @@
                   <c:v>3.7514799999999999</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>3.5009999999999999</c:v>
+                  <c:v>3.50136</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>3.2523</c:v>
@@ -2292,7 +2292,7 @@
                   <c:v>1.4799999999999258</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.99999999999988987</c:v>
+                  <c:v>1.3600000000000279</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>2.2999999999999687</c:v>
@@ -3113,7 +3113,7 @@
                   <c:v>3.7514799999999999</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>3.5009999999999999</c:v>
+                  <c:v>3.50136</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>3.2523</c:v>
@@ -9222,11 +9222,11 @@
         <v>3.5</v>
       </c>
       <c r="B18" s="14">
-        <v>3.5009999999999999</v>
+        <v>3.50136</v>
       </c>
       <c r="D18" s="3">
         <f xml:space="preserve"> PRODUCT(B18-A18, 1000)</f>
-        <v>0.99999999999988987</v>
+        <v>1.3600000000000279</v>
       </c>
       <c r="G18">
         <v>4.3517999999999999</v>

</xml_diff>